<commit_message>
updated manuscript code and data
</commit_message>
<xml_diff>
--- a/ecology_tradesoffs_data_and_code_descriptions.xlsx
+++ b/ecology_tradesoffs_data_and_code_descriptions.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10512"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danacook/PhD Projects/Reversing Unpalatable State Shift/Ecology Submission/Data &amp; Code/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danacook/PhD Projects/Reversing Unpalatable State Shift/Scientific Reports Submission/data_and_code_v3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1AF3E50-9F59-D14E-858D-D45779052140}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{213B684A-576C-7049-8EC9-AF6F527ED627}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3080" yWindow="2060" windowWidth="28040" windowHeight="17440" xr2:uid="{9F5F6057-47DC-3944-BC3B-5E30FDF05CDB}"/>
   </bookViews>

</xml_diff>